<commit_message>
Data Updated and Fix
Fix name and added more name
</commit_message>
<xml_diff>
--- a/data.xlsx
+++ b/data.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Admin\Documents\CERTIFICATES\Martial_Arts_RMUTT_REAL_WEBSITE.xlsx_driven\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C6433597-91D7-4197-B42F-4C425B776BB7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{14762DCA-AB27-47DB-B411-D4801742EFAA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="14925" yWindow="3630" windowWidth="28800" windowHeight="15345" xr2:uid="{EB9362CE-71A0-4E0E-9498-CF329F650C4C}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{EB9362CE-71A0-4E0E-9498-CF329F650C4C}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="670" uniqueCount="230">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="678" uniqueCount="234">
   <si>
     <t>พีรติ จุติเสถียรกุล</t>
   </si>
@@ -131,9 +131,6 @@
     <t>ศราวุธ เรืองรักษ์</t>
   </si>
   <si>
-    <t>ปนะวีณ แดงอาจ</t>
-  </si>
-  <si>
     <t>ณัฐการ อมิธิดา</t>
   </si>
   <si>
@@ -308,18 +305,12 @@
     <t>ศุภวิชญ์ สายอ๋อง</t>
   </si>
   <si>
-    <t>ภูมิศักดิ์ เกือก่อยอด</t>
-  </si>
-  <si>
     <t>รัตนาวลี มณีศรีขำ</t>
   </si>
   <si>
     <t>กรกฎ ศรีสงคราม</t>
   </si>
   <si>
-    <t>จรัญญาภรณ์ กิจกาญจน์</t>
-  </si>
-  <si>
     <t>สรวิชญ์ รอดกลาง</t>
   </si>
   <si>
@@ -380,9 +371,6 @@
     <t>อริศรา สีมอ</t>
   </si>
   <si>
-    <t>บูจบุหมือแล</t>
-  </si>
-  <si>
     <t>ธนโชติ พิมพ์จันทร์</t>
   </si>
   <si>
@@ -729,6 +717,30 @@
   </si>
   <si>
     <t>walk-in</t>
+  </si>
+  <si>
+    <t>ประวีณ แดงอาจ</t>
+  </si>
+  <si>
+    <t>จรัญญาภรณ์ กิจกาญจนไพบูลย์</t>
+  </si>
+  <si>
+    <t>ภูมิศักดิ์ เกื้อก่อยอด</t>
+  </si>
+  <si>
+    <t>พันธกิจ แผ่นผา</t>
+  </si>
+  <si>
+    <t>223.png</t>
+  </si>
+  <si>
+    <t>อภิเชษฐ์ วงค์แก้ว</t>
+  </si>
+  <si>
+    <t>224.png</t>
+  </si>
+  <si>
+    <t>บูจุบ หมื่อแล</t>
   </si>
 </sst>
 </file>
@@ -1116,7 +1128,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{ED36FB80-C13C-4796-91C3-FF1493E74781}">
-  <dimension ref="A1:D223"/>
+  <dimension ref="A1:D225"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="27.5703125" customWidth="1"/>
@@ -1126,16 +1138,16 @@
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>174</v>
+        <v>170</v>
       </c>
       <c r="B1" s="1" t="s">
+        <v>171</v>
+      </c>
+      <c r="C1" t="s">
+        <v>172</v>
+      </c>
+      <c r="D1" t="s">
         <v>175</v>
-      </c>
-      <c r="C1" t="s">
-        <v>176</v>
-      </c>
-      <c r="D1" t="s">
-        <v>179</v>
       </c>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.25">
@@ -1143,10 +1155,10 @@
         <v>0</v>
       </c>
       <c r="B2" t="s">
-        <v>173</v>
+        <v>169</v>
       </c>
       <c r="C2" t="s">
-        <v>177</v>
+        <v>173</v>
       </c>
       <c r="D2" t="str">
         <f>ROW(A1)&amp;".png"</f>
@@ -1158,10 +1170,10 @@
         <v>1</v>
       </c>
       <c r="B3" t="s">
-        <v>173</v>
+        <v>169</v>
       </c>
       <c r="C3" t="s">
-        <v>177</v>
+        <v>173</v>
       </c>
       <c r="D3" t="str">
         <f t="shared" ref="D3:D66" si="0">ROW(A2)&amp;".png"</f>
@@ -1173,10 +1185,10 @@
         <v>2</v>
       </c>
       <c r="B4" t="s">
-        <v>173</v>
+        <v>169</v>
       </c>
       <c r="C4" t="s">
-        <v>178</v>
+        <v>174</v>
       </c>
       <c r="D4" t="str">
         <f t="shared" si="0"/>
@@ -1188,10 +1200,10 @@
         <v>3</v>
       </c>
       <c r="B5" t="s">
-        <v>173</v>
+        <v>169</v>
       </c>
       <c r="C5" t="s">
-        <v>178</v>
+        <v>174</v>
       </c>
       <c r="D5" t="str">
         <f t="shared" si="0"/>
@@ -1203,10 +1215,10 @@
         <v>4</v>
       </c>
       <c r="B6" t="s">
-        <v>173</v>
+        <v>169</v>
       </c>
       <c r="C6" t="s">
-        <v>178</v>
+        <v>174</v>
       </c>
       <c r="D6" t="str">
         <f t="shared" si="0"/>
@@ -1218,10 +1230,10 @@
         <v>5</v>
       </c>
       <c r="B7" t="s">
-        <v>173</v>
+        <v>169</v>
       </c>
       <c r="C7" t="s">
-        <v>177</v>
+        <v>173</v>
       </c>
       <c r="D7" t="str">
         <f t="shared" si="0"/>
@@ -1233,10 +1245,10 @@
         <v>6</v>
       </c>
       <c r="B8" t="s">
-        <v>173</v>
+        <v>169</v>
       </c>
       <c r="C8" t="s">
-        <v>178</v>
+        <v>174</v>
       </c>
       <c r="D8" t="str">
         <f t="shared" si="0"/>
@@ -1248,10 +1260,10 @@
         <v>7</v>
       </c>
       <c r="B9" t="s">
-        <v>173</v>
+        <v>169</v>
       </c>
       <c r="C9" t="s">
-        <v>177</v>
+        <v>173</v>
       </c>
       <c r="D9" t="str">
         <f t="shared" si="0"/>
@@ -1263,10 +1275,10 @@
         <v>8</v>
       </c>
       <c r="B10" t="s">
-        <v>173</v>
+        <v>169</v>
       </c>
       <c r="C10" t="s">
-        <v>178</v>
+        <v>174</v>
       </c>
       <c r="D10" t="str">
         <f t="shared" si="0"/>
@@ -1278,10 +1290,10 @@
         <v>9</v>
       </c>
       <c r="B11" t="s">
-        <v>173</v>
+        <v>169</v>
       </c>
       <c r="C11" t="s">
-        <v>177</v>
+        <v>173</v>
       </c>
       <c r="D11" t="str">
         <f t="shared" si="0"/>
@@ -1293,10 +1305,10 @@
         <v>10</v>
       </c>
       <c r="B12" t="s">
-        <v>173</v>
+        <v>169</v>
       </c>
       <c r="C12" t="s">
-        <v>177</v>
+        <v>173</v>
       </c>
       <c r="D12" t="str">
         <f t="shared" si="0"/>
@@ -1308,10 +1320,10 @@
         <v>11</v>
       </c>
       <c r="B13" t="s">
-        <v>173</v>
+        <v>169</v>
       </c>
       <c r="C13" t="s">
-        <v>178</v>
+        <v>174</v>
       </c>
       <c r="D13" t="str">
         <f t="shared" si="0"/>
@@ -1323,10 +1335,10 @@
         <v>12</v>
       </c>
       <c r="B14" t="s">
-        <v>173</v>
+        <v>169</v>
       </c>
       <c r="C14" t="s">
-        <v>178</v>
+        <v>174</v>
       </c>
       <c r="D14" t="str">
         <f t="shared" si="0"/>
@@ -1338,10 +1350,10 @@
         <v>13</v>
       </c>
       <c r="B15" t="s">
-        <v>173</v>
+        <v>169</v>
       </c>
       <c r="C15" t="s">
-        <v>178</v>
+        <v>174</v>
       </c>
       <c r="D15" t="str">
         <f t="shared" si="0"/>
@@ -1353,10 +1365,10 @@
         <v>14</v>
       </c>
       <c r="B16" t="s">
-        <v>173</v>
+        <v>169</v>
       </c>
       <c r="C16" t="s">
-        <v>178</v>
+        <v>174</v>
       </c>
       <c r="D16" t="str">
         <f t="shared" si="0"/>
@@ -1368,10 +1380,10 @@
         <v>15</v>
       </c>
       <c r="B17" t="s">
-        <v>173</v>
+        <v>169</v>
       </c>
       <c r="C17" t="s">
-        <v>178</v>
+        <v>174</v>
       </c>
       <c r="D17" t="str">
         <f t="shared" si="0"/>
@@ -1383,10 +1395,10 @@
         <v>16</v>
       </c>
       <c r="B18" t="s">
-        <v>173</v>
+        <v>169</v>
       </c>
       <c r="C18" t="s">
-        <v>178</v>
+        <v>174</v>
       </c>
       <c r="D18" t="str">
         <f t="shared" si="0"/>
@@ -1398,10 +1410,10 @@
         <v>17</v>
       </c>
       <c r="B19" t="s">
-        <v>173</v>
+        <v>169</v>
       </c>
       <c r="C19" t="s">
-        <v>177</v>
+        <v>173</v>
       </c>
       <c r="D19" t="str">
         <f t="shared" si="0"/>
@@ -1413,10 +1425,10 @@
         <v>18</v>
       </c>
       <c r="B20" t="s">
-        <v>173</v>
+        <v>169</v>
       </c>
       <c r="C20" t="s">
-        <v>178</v>
+        <v>174</v>
       </c>
       <c r="D20" t="str">
         <f t="shared" si="0"/>
@@ -1428,10 +1440,10 @@
         <v>19</v>
       </c>
       <c r="B21" t="s">
-        <v>173</v>
+        <v>169</v>
       </c>
       <c r="C21" t="s">
-        <v>178</v>
+        <v>174</v>
       </c>
       <c r="D21" t="str">
         <f t="shared" si="0"/>
@@ -1443,10 +1455,10 @@
         <v>20</v>
       </c>
       <c r="B22" t="s">
-        <v>173</v>
+        <v>169</v>
       </c>
       <c r="C22" t="s">
-        <v>177</v>
+        <v>173</v>
       </c>
       <c r="D22" t="str">
         <f t="shared" si="0"/>
@@ -1458,10 +1470,10 @@
         <v>21</v>
       </c>
       <c r="B23" t="s">
-        <v>173</v>
+        <v>169</v>
       </c>
       <c r="C23" t="s">
-        <v>178</v>
+        <v>174</v>
       </c>
       <c r="D23" t="str">
         <f t="shared" si="0"/>
@@ -1473,10 +1485,10 @@
         <v>22</v>
       </c>
       <c r="B24" t="s">
-        <v>173</v>
+        <v>169</v>
       </c>
       <c r="C24" t="s">
-        <v>178</v>
+        <v>174</v>
       </c>
       <c r="D24" t="str">
         <f t="shared" si="0"/>
@@ -1488,10 +1500,10 @@
         <v>23</v>
       </c>
       <c r="B25" t="s">
-        <v>173</v>
+        <v>169</v>
       </c>
       <c r="C25" t="s">
-        <v>178</v>
+        <v>174</v>
       </c>
       <c r="D25" t="str">
         <f t="shared" si="0"/>
@@ -1503,10 +1515,10 @@
         <v>24</v>
       </c>
       <c r="B26" t="s">
-        <v>173</v>
+        <v>169</v>
       </c>
       <c r="C26" t="s">
-        <v>177</v>
+        <v>173</v>
       </c>
       <c r="D26" t="str">
         <f t="shared" si="0"/>
@@ -1518,10 +1530,10 @@
         <v>25</v>
       </c>
       <c r="B27" t="s">
-        <v>173</v>
+        <v>169</v>
       </c>
       <c r="C27" t="s">
-        <v>178</v>
+        <v>174</v>
       </c>
       <c r="D27" t="str">
         <f t="shared" si="0"/>
@@ -1533,10 +1545,10 @@
         <v>26</v>
       </c>
       <c r="B28" t="s">
-        <v>173</v>
+        <v>169</v>
       </c>
       <c r="C28" t="s">
-        <v>178</v>
+        <v>174</v>
       </c>
       <c r="D28" t="str">
         <f t="shared" si="0"/>
@@ -1548,10 +1560,10 @@
         <v>27</v>
       </c>
       <c r="B29" t="s">
-        <v>173</v>
+        <v>169</v>
       </c>
       <c r="C29" t="s">
-        <v>178</v>
+        <v>174</v>
       </c>
       <c r="D29" t="str">
         <f t="shared" si="0"/>
@@ -1563,10 +1575,10 @@
         <v>28</v>
       </c>
       <c r="B30" t="s">
-        <v>173</v>
+        <v>169</v>
       </c>
       <c r="C30" t="s">
-        <v>178</v>
+        <v>174</v>
       </c>
       <c r="D30" t="str">
         <f t="shared" si="0"/>
@@ -1578,10 +1590,10 @@
         <v>29</v>
       </c>
       <c r="B31" t="s">
-        <v>173</v>
+        <v>169</v>
       </c>
       <c r="C31" t="s">
-        <v>178</v>
+        <v>174</v>
       </c>
       <c r="D31" t="str">
         <f t="shared" si="0"/>
@@ -1590,13 +1602,13 @@
     </row>
     <row r="32" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
-        <v>30</v>
+        <v>226</v>
       </c>
       <c r="B32" t="s">
-        <v>173</v>
+        <v>169</v>
       </c>
       <c r="C32" t="s">
-        <v>177</v>
+        <v>173</v>
       </c>
       <c r="D32" t="str">
         <f t="shared" si="0"/>
@@ -1605,13 +1617,13 @@
     </row>
     <row r="33" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="B33" t="s">
-        <v>173</v>
+        <v>169</v>
       </c>
       <c r="C33" t="s">
-        <v>178</v>
+        <v>174</v>
       </c>
       <c r="D33" t="str">
         <f t="shared" si="0"/>
@@ -1620,13 +1632,13 @@
     </row>
     <row r="34" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="B34" t="s">
-        <v>173</v>
+        <v>169</v>
       </c>
       <c r="C34" t="s">
-        <v>178</v>
+        <v>174</v>
       </c>
       <c r="D34" t="str">
         <f t="shared" si="0"/>
@@ -1635,13 +1647,13 @@
     </row>
     <row r="35" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="B35" t="s">
-        <v>173</v>
+        <v>169</v>
       </c>
       <c r="C35" t="s">
-        <v>178</v>
+        <v>174</v>
       </c>
       <c r="D35" t="str">
         <f t="shared" si="0"/>
@@ -1650,13 +1662,13 @@
     </row>
     <row r="36" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A36" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="B36" t="s">
-        <v>173</v>
+        <v>169</v>
       </c>
       <c r="C36" t="s">
-        <v>178</v>
+        <v>174</v>
       </c>
       <c r="D36" t="str">
         <f t="shared" si="0"/>
@@ -1665,13 +1677,13 @@
     </row>
     <row r="37" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A37" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="B37" t="s">
-        <v>173</v>
+        <v>169</v>
       </c>
       <c r="C37" t="s">
-        <v>177</v>
+        <v>173</v>
       </c>
       <c r="D37" t="str">
         <f t="shared" si="0"/>
@@ -1680,13 +1692,13 @@
     </row>
     <row r="38" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A38" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="B38" t="s">
-        <v>173</v>
+        <v>169</v>
       </c>
       <c r="C38" t="s">
-        <v>177</v>
+        <v>173</v>
       </c>
       <c r="D38" t="str">
         <f t="shared" si="0"/>
@@ -1695,13 +1707,13 @@
     </row>
     <row r="39" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A39" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="B39" t="s">
-        <v>173</v>
+        <v>169</v>
       </c>
       <c r="C39" t="s">
-        <v>178</v>
+        <v>174</v>
       </c>
       <c r="D39" t="str">
         <f t="shared" si="0"/>
@@ -1710,13 +1722,13 @@
     </row>
     <row r="40" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A40" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="B40" t="s">
-        <v>173</v>
+        <v>169</v>
       </c>
       <c r="C40" t="s">
-        <v>178</v>
+        <v>174</v>
       </c>
       <c r="D40" t="str">
         <f t="shared" si="0"/>
@@ -1725,13 +1737,13 @@
     </row>
     <row r="41" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A41" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="B41" t="s">
-        <v>173</v>
+        <v>169</v>
       </c>
       <c r="C41" t="s">
-        <v>177</v>
+        <v>173</v>
       </c>
       <c r="D41" t="str">
         <f t="shared" si="0"/>
@@ -1740,13 +1752,13 @@
     </row>
     <row r="42" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A42" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="B42" t="s">
-        <v>173</v>
+        <v>169</v>
       </c>
       <c r="C42" t="s">
-        <v>178</v>
+        <v>174</v>
       </c>
       <c r="D42" t="str">
         <f t="shared" si="0"/>
@@ -1755,13 +1767,13 @@
     </row>
     <row r="43" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A43" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="B43" t="s">
-        <v>173</v>
+        <v>169</v>
       </c>
       <c r="C43" t="s">
-        <v>178</v>
+        <v>174</v>
       </c>
       <c r="D43" t="str">
         <f t="shared" si="0"/>
@@ -1770,13 +1782,13 @@
     </row>
     <row r="44" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A44" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="B44" t="s">
-        <v>173</v>
+        <v>169</v>
       </c>
       <c r="C44" t="s">
-        <v>177</v>
+        <v>173</v>
       </c>
       <c r="D44" t="str">
         <f t="shared" si="0"/>
@@ -1785,13 +1797,13 @@
     </row>
     <row r="45" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A45" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="B45" t="s">
-        <v>173</v>
+        <v>169</v>
       </c>
       <c r="C45" t="s">
-        <v>178</v>
+        <v>174</v>
       </c>
       <c r="D45" t="str">
         <f t="shared" si="0"/>
@@ -1800,13 +1812,13 @@
     </row>
     <row r="46" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A46" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="B46" t="s">
-        <v>173</v>
+        <v>169</v>
       </c>
       <c r="C46" t="s">
-        <v>178</v>
+        <v>174</v>
       </c>
       <c r="D46" t="str">
         <f t="shared" si="0"/>
@@ -1815,13 +1827,13 @@
     </row>
     <row r="47" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A47" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="B47" t="s">
-        <v>173</v>
+        <v>169</v>
       </c>
       <c r="C47" t="s">
-        <v>178</v>
+        <v>174</v>
       </c>
       <c r="D47" t="str">
         <f t="shared" si="0"/>
@@ -1830,13 +1842,13 @@
     </row>
     <row r="48" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A48" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="B48" t="s">
-        <v>173</v>
+        <v>169</v>
       </c>
       <c r="C48" t="s">
-        <v>178</v>
+        <v>173</v>
       </c>
       <c r="D48" t="str">
         <f t="shared" si="0"/>
@@ -1845,13 +1857,13 @@
     </row>
     <row r="49" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A49" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="B49" t="s">
-        <v>173</v>
+        <v>169</v>
       </c>
       <c r="C49" t="s">
-        <v>178</v>
+        <v>174</v>
       </c>
       <c r="D49" t="str">
         <f t="shared" si="0"/>
@@ -1860,13 +1872,13 @@
     </row>
     <row r="50" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A50" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="B50" t="s">
-        <v>173</v>
+        <v>169</v>
       </c>
       <c r="C50" t="s">
-        <v>178</v>
+        <v>174</v>
       </c>
       <c r="D50" t="str">
         <f t="shared" si="0"/>
@@ -1875,13 +1887,13 @@
     </row>
     <row r="51" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A51" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="B51" t="s">
-        <v>173</v>
+        <v>169</v>
       </c>
       <c r="C51" t="s">
-        <v>177</v>
+        <v>173</v>
       </c>
       <c r="D51" t="str">
         <f t="shared" si="0"/>
@@ -1890,13 +1902,13 @@
     </row>
     <row r="52" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A52" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="B52" t="s">
-        <v>173</v>
+        <v>169</v>
       </c>
       <c r="C52" t="s">
-        <v>178</v>
+        <v>174</v>
       </c>
       <c r="D52" t="str">
         <f t="shared" si="0"/>
@@ -1905,13 +1917,13 @@
     </row>
     <row r="53" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A53" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="B53" t="s">
-        <v>173</v>
+        <v>169</v>
       </c>
       <c r="C53" t="s">
-        <v>178</v>
+        <v>174</v>
       </c>
       <c r="D53" t="str">
         <f t="shared" si="0"/>
@@ -1920,13 +1932,13 @@
     </row>
     <row r="54" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A54" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="B54" t="s">
-        <v>173</v>
+        <v>169</v>
       </c>
       <c r="C54" t="s">
-        <v>177</v>
+        <v>173</v>
       </c>
       <c r="D54" t="str">
         <f t="shared" si="0"/>
@@ -1935,13 +1947,13 @@
     </row>
     <row r="55" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A55" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="B55" t="s">
-        <v>173</v>
+        <v>169</v>
       </c>
       <c r="C55" t="s">
-        <v>178</v>
+        <v>174</v>
       </c>
       <c r="D55" t="str">
         <f t="shared" si="0"/>
@@ -1950,13 +1962,13 @@
     </row>
     <row r="56" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A56" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="B56" t="s">
-        <v>173</v>
+        <v>169</v>
       </c>
       <c r="C56" t="s">
-        <v>178</v>
+        <v>174</v>
       </c>
       <c r="D56" t="str">
         <f t="shared" si="0"/>
@@ -1965,13 +1977,13 @@
     </row>
     <row r="57" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A57" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="B57" t="s">
-        <v>173</v>
+        <v>169</v>
       </c>
       <c r="C57" t="s">
-        <v>177</v>
+        <v>173</v>
       </c>
       <c r="D57" t="str">
         <f t="shared" si="0"/>
@@ -1980,13 +1992,13 @@
     </row>
     <row r="58" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A58" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="B58" t="s">
-        <v>173</v>
+        <v>169</v>
       </c>
       <c r="C58" t="s">
-        <v>177</v>
+        <v>173</v>
       </c>
       <c r="D58" t="str">
         <f t="shared" si="0"/>
@@ -1995,13 +2007,13 @@
     </row>
     <row r="59" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A59" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="B59" t="s">
-        <v>173</v>
+        <v>169</v>
       </c>
       <c r="C59" t="s">
-        <v>178</v>
+        <v>174</v>
       </c>
       <c r="D59" t="str">
         <f t="shared" si="0"/>
@@ -2010,13 +2022,13 @@
     </row>
     <row r="60" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A60" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="B60" t="s">
-        <v>173</v>
+        <v>169</v>
       </c>
       <c r="C60" t="s">
-        <v>177</v>
+        <v>173</v>
       </c>
       <c r="D60" t="str">
         <f t="shared" si="0"/>
@@ -2025,13 +2037,13 @@
     </row>
     <row r="61" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A61" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="B61" t="s">
-        <v>173</v>
+        <v>169</v>
       </c>
       <c r="C61" t="s">
-        <v>178</v>
+        <v>174</v>
       </c>
       <c r="D61" t="str">
         <f t="shared" si="0"/>
@@ -2040,13 +2052,13 @@
     </row>
     <row r="62" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A62" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="B62" t="s">
-        <v>173</v>
+        <v>169</v>
       </c>
       <c r="C62" t="s">
-        <v>177</v>
+        <v>173</v>
       </c>
       <c r="D62" t="str">
         <f t="shared" si="0"/>
@@ -2055,13 +2067,13 @@
     </row>
     <row r="63" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A63" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="B63" t="s">
-        <v>173</v>
+        <v>169</v>
       </c>
       <c r="C63" t="s">
-        <v>178</v>
+        <v>174</v>
       </c>
       <c r="D63" t="str">
         <f t="shared" si="0"/>
@@ -2070,13 +2082,13 @@
     </row>
     <row r="64" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A64" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="B64" t="s">
-        <v>173</v>
+        <v>169</v>
       </c>
       <c r="C64" t="s">
-        <v>178</v>
+        <v>174</v>
       </c>
       <c r="D64" t="str">
         <f t="shared" si="0"/>
@@ -2085,13 +2097,13 @@
     </row>
     <row r="65" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A65" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="B65" t="s">
-        <v>173</v>
+        <v>169</v>
       </c>
       <c r="C65" t="s">
-        <v>178</v>
+        <v>174</v>
       </c>
       <c r="D65" t="str">
         <f t="shared" si="0"/>
@@ -2100,13 +2112,13 @@
     </row>
     <row r="66" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A66" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="B66" t="s">
-        <v>173</v>
+        <v>169</v>
       </c>
       <c r="C66" t="s">
-        <v>178</v>
+        <v>174</v>
       </c>
       <c r="D66" t="str">
         <f t="shared" si="0"/>
@@ -2115,13 +2127,13 @@
     </row>
     <row r="67" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A67" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="B67" t="s">
-        <v>173</v>
+        <v>169</v>
       </c>
       <c r="C67" t="s">
-        <v>177</v>
+        <v>173</v>
       </c>
       <c r="D67" t="str">
         <f t="shared" ref="D67:D130" si="1">ROW(A66)&amp;".png"</f>
@@ -2130,13 +2142,13 @@
     </row>
     <row r="68" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A68" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="B68" t="s">
-        <v>173</v>
+        <v>169</v>
       </c>
       <c r="C68" t="s">
-        <v>178</v>
+        <v>174</v>
       </c>
       <c r="D68" t="str">
         <f t="shared" si="1"/>
@@ -2145,13 +2157,13 @@
     </row>
     <row r="69" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A69" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="B69" t="s">
-        <v>173</v>
+        <v>169</v>
       </c>
       <c r="C69" t="s">
-        <v>177</v>
+        <v>173</v>
       </c>
       <c r="D69" t="str">
         <f t="shared" si="1"/>
@@ -2160,13 +2172,13 @@
     </row>
     <row r="70" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A70" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="B70" t="s">
-        <v>173</v>
+        <v>169</v>
       </c>
       <c r="C70" t="s">
-        <v>178</v>
+        <v>174</v>
       </c>
       <c r="D70" t="str">
         <f t="shared" si="1"/>
@@ -2175,13 +2187,13 @@
     </row>
     <row r="71" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A71" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="B71" t="s">
-        <v>173</v>
+        <v>169</v>
       </c>
       <c r="C71" t="s">
-        <v>177</v>
+        <v>173</v>
       </c>
       <c r="D71" t="str">
         <f t="shared" si="1"/>
@@ -2190,13 +2202,13 @@
     </row>
     <row r="72" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A72" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="B72" t="s">
-        <v>173</v>
+        <v>169</v>
       </c>
       <c r="C72" t="s">
-        <v>178</v>
+        <v>174</v>
       </c>
       <c r="D72" t="str">
         <f t="shared" si="1"/>
@@ -2205,13 +2217,13 @@
     </row>
     <row r="73" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A73" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="B73" t="s">
-        <v>173</v>
+        <v>169</v>
       </c>
       <c r="C73" t="s">
-        <v>178</v>
+        <v>174</v>
       </c>
       <c r="D73" t="str">
         <f t="shared" si="1"/>
@@ -2220,13 +2232,13 @@
     </row>
     <row r="74" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A74" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="B74" t="s">
-        <v>173</v>
+        <v>169</v>
       </c>
       <c r="C74" t="s">
-        <v>178</v>
+        <v>174</v>
       </c>
       <c r="D74" t="str">
         <f t="shared" si="1"/>
@@ -2235,13 +2247,13 @@
     </row>
     <row r="75" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A75" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="B75" t="s">
-        <v>173</v>
+        <v>169</v>
       </c>
       <c r="C75" t="s">
-        <v>178</v>
+        <v>174</v>
       </c>
       <c r="D75" t="str">
         <f t="shared" si="1"/>
@@ -2250,13 +2262,13 @@
     </row>
     <row r="76" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A76" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="B76" t="s">
-        <v>173</v>
+        <v>169</v>
       </c>
       <c r="C76" t="s">
-        <v>177</v>
+        <v>173</v>
       </c>
       <c r="D76" t="str">
         <f t="shared" si="1"/>
@@ -2265,13 +2277,13 @@
     </row>
     <row r="77" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A77" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="B77" t="s">
-        <v>173</v>
+        <v>169</v>
       </c>
       <c r="C77" t="s">
-        <v>178</v>
+        <v>174</v>
       </c>
       <c r="D77" t="str">
         <f t="shared" si="1"/>
@@ -2280,13 +2292,13 @@
     </row>
     <row r="78" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A78" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="B78" t="s">
-        <v>173</v>
+        <v>169</v>
       </c>
       <c r="C78" t="s">
-        <v>177</v>
+        <v>173</v>
       </c>
       <c r="D78" t="str">
         <f t="shared" si="1"/>
@@ -2295,13 +2307,13 @@
     </row>
     <row r="79" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A79" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="B79" t="s">
-        <v>173</v>
+        <v>169</v>
       </c>
       <c r="C79" t="s">
-        <v>177</v>
+        <v>173</v>
       </c>
       <c r="D79" t="str">
         <f t="shared" si="1"/>
@@ -2310,13 +2322,13 @@
     </row>
     <row r="80" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A80" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="B80" t="s">
-        <v>173</v>
+        <v>169</v>
       </c>
       <c r="C80" t="s">
-        <v>178</v>
+        <v>174</v>
       </c>
       <c r="D80" t="str">
         <f t="shared" si="1"/>
@@ -2325,13 +2337,13 @@
     </row>
     <row r="81" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A81" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="B81" t="s">
-        <v>173</v>
+        <v>169</v>
       </c>
       <c r="C81" t="s">
-        <v>177</v>
+        <v>173</v>
       </c>
       <c r="D81" t="str">
         <f t="shared" si="1"/>
@@ -2340,13 +2352,13 @@
     </row>
     <row r="82" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A82" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="B82" t="s">
-        <v>173</v>
+        <v>169</v>
       </c>
       <c r="C82" t="s">
-        <v>178</v>
+        <v>174</v>
       </c>
       <c r="D82" t="str">
         <f t="shared" si="1"/>
@@ -2355,13 +2367,13 @@
     </row>
     <row r="83" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A83" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="B83" t="s">
-        <v>173</v>
+        <v>169</v>
       </c>
       <c r="C83" t="s">
-        <v>178</v>
+        <v>174</v>
       </c>
       <c r="D83" t="str">
         <f t="shared" si="1"/>
@@ -2370,13 +2382,13 @@
     </row>
     <row r="84" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A84" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="B84" t="s">
-        <v>173</v>
+        <v>169</v>
       </c>
       <c r="C84" t="s">
-        <v>177</v>
+        <v>173</v>
       </c>
       <c r="D84" t="str">
         <f t="shared" si="1"/>
@@ -2385,13 +2397,13 @@
     </row>
     <row r="85" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A85" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="B85" t="s">
-        <v>173</v>
+        <v>169</v>
       </c>
       <c r="C85" t="s">
-        <v>177</v>
+        <v>173</v>
       </c>
       <c r="D85" t="str">
         <f t="shared" si="1"/>
@@ -2400,13 +2412,13 @@
     </row>
     <row r="86" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A86" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="B86" t="s">
-        <v>173</v>
+        <v>169</v>
       </c>
       <c r="C86" t="s">
-        <v>178</v>
+        <v>174</v>
       </c>
       <c r="D86" t="str">
         <f t="shared" si="1"/>
@@ -2415,13 +2427,13 @@
     </row>
     <row r="87" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A87" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="B87" t="s">
-        <v>173</v>
+        <v>169</v>
       </c>
       <c r="C87" t="s">
-        <v>178</v>
+        <v>174</v>
       </c>
       <c r="D87" t="str">
         <f t="shared" si="1"/>
@@ -2430,13 +2442,13 @@
     </row>
     <row r="88" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A88" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="B88" t="s">
-        <v>173</v>
+        <v>169</v>
       </c>
       <c r="C88" t="s">
-        <v>178</v>
+        <v>174</v>
       </c>
       <c r="D88" t="str">
         <f t="shared" si="1"/>
@@ -2445,13 +2457,13 @@
     </row>
     <row r="89" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A89" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="B89" t="s">
-        <v>173</v>
+        <v>169</v>
       </c>
       <c r="C89" t="s">
-        <v>177</v>
+        <v>173</v>
       </c>
       <c r="D89" t="str">
         <f t="shared" si="1"/>
@@ -2460,13 +2472,13 @@
     </row>
     <row r="90" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A90" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="B90" t="s">
-        <v>173</v>
+        <v>169</v>
       </c>
       <c r="C90" t="s">
-        <v>178</v>
+        <v>174</v>
       </c>
       <c r="D90" t="str">
         <f t="shared" si="1"/>
@@ -2475,13 +2487,13 @@
     </row>
     <row r="91" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A91" t="s">
-        <v>89</v>
+        <v>228</v>
       </c>
       <c r="B91" t="s">
-        <v>173</v>
+        <v>169</v>
       </c>
       <c r="C91" t="s">
-        <v>177</v>
+        <v>173</v>
       </c>
       <c r="D91" t="str">
         <f t="shared" si="1"/>
@@ -2490,13 +2502,13 @@
     </row>
     <row r="92" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A92" t="s">
-        <v>90</v>
+        <v>88</v>
       </c>
       <c r="B92" t="s">
-        <v>173</v>
+        <v>169</v>
       </c>
       <c r="C92" t="s">
-        <v>178</v>
+        <v>174</v>
       </c>
       <c r="D92" t="str">
         <f t="shared" si="1"/>
@@ -2505,13 +2517,13 @@
     </row>
     <row r="93" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A93" t="s">
-        <v>91</v>
+        <v>89</v>
       </c>
       <c r="B93" t="s">
-        <v>173</v>
+        <v>169</v>
       </c>
       <c r="C93" t="s">
-        <v>178</v>
+        <v>174</v>
       </c>
       <c r="D93" t="str">
         <f t="shared" si="1"/>
@@ -2520,13 +2532,13 @@
     </row>
     <row r="94" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A94" t="s">
-        <v>92</v>
+        <v>227</v>
       </c>
       <c r="B94" t="s">
-        <v>173</v>
+        <v>169</v>
       </c>
       <c r="C94" t="s">
-        <v>177</v>
+        <v>173</v>
       </c>
       <c r="D94" t="str">
         <f t="shared" si="1"/>
@@ -2535,13 +2547,13 @@
     </row>
     <row r="95" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A95" t="s">
-        <v>93</v>
+        <v>90</v>
       </c>
       <c r="B95" t="s">
-        <v>173</v>
+        <v>169</v>
       </c>
       <c r="C95" t="s">
-        <v>177</v>
+        <v>173</v>
       </c>
       <c r="D95" t="str">
         <f t="shared" si="1"/>
@@ -2550,13 +2562,13 @@
     </row>
     <row r="96" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A96" t="s">
-        <v>94</v>
+        <v>91</v>
       </c>
       <c r="B96" t="s">
-        <v>173</v>
+        <v>169</v>
       </c>
       <c r="C96" t="s">
-        <v>178</v>
+        <v>174</v>
       </c>
       <c r="D96" t="str">
         <f t="shared" si="1"/>
@@ -2565,13 +2577,13 @@
     </row>
     <row r="97" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A97" t="s">
-        <v>95</v>
+        <v>92</v>
       </c>
       <c r="B97" t="s">
-        <v>173</v>
+        <v>169</v>
       </c>
       <c r="C97" t="s">
-        <v>177</v>
+        <v>173</v>
       </c>
       <c r="D97" t="str">
         <f t="shared" si="1"/>
@@ -2580,13 +2592,13 @@
     </row>
     <row r="98" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A98" t="s">
-        <v>96</v>
+        <v>93</v>
       </c>
       <c r="B98" t="s">
-        <v>173</v>
+        <v>169</v>
       </c>
       <c r="C98" t="s">
-        <v>178</v>
+        <v>174</v>
       </c>
       <c r="D98" t="str">
         <f t="shared" si="1"/>
@@ -2595,13 +2607,13 @@
     </row>
     <row r="99" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A99" t="s">
-        <v>97</v>
+        <v>94</v>
       </c>
       <c r="B99" t="s">
-        <v>173</v>
+        <v>169</v>
       </c>
       <c r="C99" t="s">
-        <v>178</v>
+        <v>174</v>
       </c>
       <c r="D99" t="str">
         <f t="shared" si="1"/>
@@ -2610,13 +2622,13 @@
     </row>
     <row r="100" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A100" t="s">
-        <v>98</v>
+        <v>95</v>
       </c>
       <c r="B100" t="s">
-        <v>173</v>
+        <v>169</v>
       </c>
       <c r="C100" t="s">
-        <v>177</v>
+        <v>173</v>
       </c>
       <c r="D100" t="str">
         <f t="shared" si="1"/>
@@ -2625,13 +2637,13 @@
     </row>
     <row r="101" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A101" t="s">
-        <v>99</v>
+        <v>96</v>
       </c>
       <c r="B101" t="s">
-        <v>173</v>
+        <v>169</v>
       </c>
       <c r="C101" t="s">
-        <v>177</v>
+        <v>173</v>
       </c>
       <c r="D101" t="str">
         <f t="shared" si="1"/>
@@ -2640,13 +2652,13 @@
     </row>
     <row r="102" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A102" t="s">
-        <v>100</v>
+        <v>97</v>
       </c>
       <c r="B102" t="s">
-        <v>173</v>
+        <v>169</v>
       </c>
       <c r="C102" t="s">
-        <v>178</v>
+        <v>174</v>
       </c>
       <c r="D102" t="str">
         <f t="shared" si="1"/>
@@ -2655,13 +2667,13 @@
     </row>
     <row r="103" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A103" t="s">
-        <v>101</v>
+        <v>98</v>
       </c>
       <c r="B103" t="s">
-        <v>173</v>
+        <v>169</v>
       </c>
       <c r="C103" t="s">
-        <v>177</v>
+        <v>173</v>
       </c>
       <c r="D103" t="str">
         <f t="shared" si="1"/>
@@ -2670,13 +2682,13 @@
     </row>
     <row r="104" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A104" t="s">
-        <v>102</v>
+        <v>99</v>
       </c>
       <c r="B104" t="s">
-        <v>173</v>
+        <v>169</v>
       </c>
       <c r="C104" t="s">
-        <v>178</v>
+        <v>174</v>
       </c>
       <c r="D104" t="str">
         <f t="shared" si="1"/>
@@ -2685,13 +2697,13 @@
     </row>
     <row r="105" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A105" t="s">
-        <v>103</v>
+        <v>100</v>
       </c>
       <c r="B105" t="s">
-        <v>173</v>
+        <v>169</v>
       </c>
       <c r="C105" t="s">
-        <v>177</v>
+        <v>173</v>
       </c>
       <c r="D105" t="str">
         <f t="shared" si="1"/>
@@ -2700,13 +2712,13 @@
     </row>
     <row r="106" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A106" t="s">
-        <v>104</v>
+        <v>101</v>
       </c>
       <c r="B106" t="s">
-        <v>173</v>
+        <v>169</v>
       </c>
       <c r="C106" t="s">
-        <v>178</v>
+        <v>174</v>
       </c>
       <c r="D106" t="str">
         <f t="shared" si="1"/>
@@ -2715,13 +2727,13 @@
     </row>
     <row r="107" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A107" t="s">
-        <v>105</v>
+        <v>102</v>
       </c>
       <c r="B107" t="s">
-        <v>173</v>
+        <v>169</v>
       </c>
       <c r="C107" t="s">
-        <v>178</v>
+        <v>174</v>
       </c>
       <c r="D107" t="str">
         <f t="shared" si="1"/>
@@ -2730,13 +2742,13 @@
     </row>
     <row r="108" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A108" t="s">
-        <v>106</v>
+        <v>103</v>
       </c>
       <c r="B108" t="s">
-        <v>173</v>
+        <v>169</v>
       </c>
       <c r="C108" t="s">
-        <v>177</v>
+        <v>173</v>
       </c>
       <c r="D108" t="str">
         <f t="shared" si="1"/>
@@ -2745,13 +2757,13 @@
     </row>
     <row r="109" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A109" t="s">
-        <v>107</v>
+        <v>104</v>
       </c>
       <c r="B109" t="s">
-        <v>173</v>
+        <v>169</v>
       </c>
       <c r="C109" t="s">
-        <v>177</v>
+        <v>173</v>
       </c>
       <c r="D109" t="str">
         <f t="shared" si="1"/>
@@ -2760,13 +2772,13 @@
     </row>
     <row r="110" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A110" t="s">
-        <v>108</v>
+        <v>105</v>
       </c>
       <c r="B110" t="s">
-        <v>173</v>
+        <v>169</v>
       </c>
       <c r="C110" t="s">
-        <v>178</v>
+        <v>174</v>
       </c>
       <c r="D110" t="str">
         <f t="shared" si="1"/>
@@ -2775,13 +2787,13 @@
     </row>
     <row r="111" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A111" t="s">
-        <v>109</v>
+        <v>106</v>
       </c>
       <c r="B111" t="s">
-        <v>173</v>
+        <v>169</v>
       </c>
       <c r="C111" t="s">
-        <v>178</v>
+        <v>174</v>
       </c>
       <c r="D111" t="str">
         <f t="shared" si="1"/>
@@ -2790,13 +2802,13 @@
     </row>
     <row r="112" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A112" t="s">
-        <v>110</v>
+        <v>107</v>
       </c>
       <c r="B112" t="s">
-        <v>173</v>
+        <v>169</v>
       </c>
       <c r="C112" t="s">
-        <v>178</v>
+        <v>174</v>
       </c>
       <c r="D112" t="str">
         <f t="shared" si="1"/>
@@ -2805,13 +2817,13 @@
     </row>
     <row r="113" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A113" t="s">
-        <v>111</v>
+        <v>108</v>
       </c>
       <c r="B113" t="s">
-        <v>173</v>
+        <v>169</v>
       </c>
       <c r="C113" t="s">
-        <v>177</v>
+        <v>173</v>
       </c>
       <c r="D113" t="str">
         <f t="shared" si="1"/>
@@ -2820,13 +2832,13 @@
     </row>
     <row r="114" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A114" t="s">
-        <v>112</v>
+        <v>109</v>
       </c>
       <c r="B114" t="s">
-        <v>173</v>
+        <v>169</v>
       </c>
       <c r="C114" t="s">
-        <v>177</v>
+        <v>173</v>
       </c>
       <c r="D114" t="str">
         <f t="shared" si="1"/>
@@ -2835,13 +2847,13 @@
     </row>
     <row r="115" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A115" t="s">
-        <v>113</v>
+        <v>233</v>
       </c>
       <c r="B115" t="s">
-        <v>173</v>
+        <v>169</v>
       </c>
       <c r="C115" t="s">
-        <v>177</v>
+        <v>173</v>
       </c>
       <c r="D115" t="str">
         <f t="shared" si="1"/>
@@ -2850,13 +2862,13 @@
     </row>
     <row r="116" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A116" t="s">
-        <v>114</v>
+        <v>110</v>
       </c>
       <c r="B116" t="s">
-        <v>173</v>
+        <v>169</v>
       </c>
       <c r="C116" t="s">
-        <v>177</v>
+        <v>173</v>
       </c>
       <c r="D116" t="str">
         <f t="shared" si="1"/>
@@ -2865,13 +2877,13 @@
     </row>
     <row r="117" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A117" t="s">
-        <v>115</v>
+        <v>111</v>
       </c>
       <c r="B117" t="s">
-        <v>173</v>
+        <v>169</v>
       </c>
       <c r="C117" t="s">
-        <v>177</v>
+        <v>173</v>
       </c>
       <c r="D117" t="str">
         <f t="shared" si="1"/>
@@ -2880,13 +2892,13 @@
     </row>
     <row r="118" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A118" t="s">
-        <v>116</v>
+        <v>112</v>
       </c>
       <c r="B118" t="s">
-        <v>173</v>
+        <v>169</v>
       </c>
       <c r="C118" t="s">
-        <v>178</v>
+        <v>174</v>
       </c>
       <c r="D118" t="str">
         <f t="shared" si="1"/>
@@ -2895,13 +2907,13 @@
     </row>
     <row r="119" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A119" t="s">
-        <v>117</v>
+        <v>113</v>
       </c>
       <c r="B119" t="s">
-        <v>173</v>
+        <v>169</v>
       </c>
       <c r="C119" t="s">
-        <v>178</v>
+        <v>174</v>
       </c>
       <c r="D119" t="str">
         <f t="shared" si="1"/>
@@ -2910,13 +2922,13 @@
     </row>
     <row r="120" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A120" t="s">
-        <v>118</v>
+        <v>114</v>
       </c>
       <c r="B120" t="s">
-        <v>173</v>
+        <v>169</v>
       </c>
       <c r="C120" t="s">
-        <v>178</v>
+        <v>174</v>
       </c>
       <c r="D120" t="str">
         <f t="shared" si="1"/>
@@ -2925,13 +2937,13 @@
     </row>
     <row r="121" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A121" t="s">
-        <v>119</v>
+        <v>115</v>
       </c>
       <c r="B121" t="s">
-        <v>173</v>
+        <v>169</v>
       </c>
       <c r="C121" t="s">
-        <v>178</v>
+        <v>174</v>
       </c>
       <c r="D121" t="str">
         <f t="shared" si="1"/>
@@ -2940,13 +2952,13 @@
     </row>
     <row r="122" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A122" t="s">
-        <v>120</v>
+        <v>116</v>
       </c>
       <c r="B122" t="s">
-        <v>173</v>
+        <v>169</v>
       </c>
       <c r="C122" t="s">
-        <v>178</v>
+        <v>174</v>
       </c>
       <c r="D122" t="str">
         <f t="shared" si="1"/>
@@ -2955,13 +2967,13 @@
     </row>
     <row r="123" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A123" t="s">
-        <v>121</v>
+        <v>117</v>
       </c>
       <c r="B123" t="s">
-        <v>173</v>
+        <v>169</v>
       </c>
       <c r="C123" t="s">
-        <v>178</v>
+        <v>174</v>
       </c>
       <c r="D123" t="str">
         <f t="shared" si="1"/>
@@ -2970,13 +2982,13 @@
     </row>
     <row r="124" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A124" t="s">
-        <v>122</v>
+        <v>118</v>
       </c>
       <c r="B124" t="s">
-        <v>173</v>
+        <v>169</v>
       </c>
       <c r="C124" t="s">
-        <v>178</v>
+        <v>174</v>
       </c>
       <c r="D124" t="str">
         <f t="shared" si="1"/>
@@ -2985,13 +2997,13 @@
     </row>
     <row r="125" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A125" t="s">
-        <v>123</v>
+        <v>119</v>
       </c>
       <c r="B125" t="s">
-        <v>173</v>
+        <v>169</v>
       </c>
       <c r="C125" t="s">
-        <v>178</v>
+        <v>174</v>
       </c>
       <c r="D125" t="str">
         <f t="shared" si="1"/>
@@ -3000,13 +3012,13 @@
     </row>
     <row r="126" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A126" t="s">
-        <v>124</v>
+        <v>120</v>
       </c>
       <c r="B126" t="s">
-        <v>173</v>
+        <v>169</v>
       </c>
       <c r="C126" t="s">
-        <v>178</v>
+        <v>174</v>
       </c>
       <c r="D126" t="str">
         <f t="shared" si="1"/>
@@ -3015,13 +3027,13 @@
     </row>
     <row r="127" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A127" t="s">
-        <v>125</v>
+        <v>121</v>
       </c>
       <c r="B127" t="s">
-        <v>173</v>
+        <v>169</v>
       </c>
       <c r="C127" t="s">
-        <v>177</v>
+        <v>173</v>
       </c>
       <c r="D127" t="str">
         <f t="shared" si="1"/>
@@ -3030,13 +3042,13 @@
     </row>
     <row r="128" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A128" t="s">
-        <v>126</v>
+        <v>122</v>
       </c>
       <c r="B128" t="s">
-        <v>173</v>
+        <v>169</v>
       </c>
       <c r="C128" t="s">
-        <v>177</v>
+        <v>173</v>
       </c>
       <c r="D128" t="str">
         <f t="shared" si="1"/>
@@ -3045,13 +3057,13 @@
     </row>
     <row r="129" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A129" t="s">
-        <v>127</v>
+        <v>123</v>
       </c>
       <c r="B129" t="s">
-        <v>173</v>
+        <v>169</v>
       </c>
       <c r="C129" t="s">
-        <v>177</v>
+        <v>173</v>
       </c>
       <c r="D129" t="str">
         <f t="shared" si="1"/>
@@ -3060,13 +3072,13 @@
     </row>
     <row r="130" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A130" t="s">
-        <v>128</v>
+        <v>124</v>
       </c>
       <c r="B130" t="s">
-        <v>173</v>
+        <v>169</v>
       </c>
       <c r="C130" t="s">
-        <v>177</v>
+        <v>173</v>
       </c>
       <c r="D130" t="str">
         <f t="shared" si="1"/>
@@ -3075,13 +3087,13 @@
     </row>
     <row r="131" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A131" t="s">
-        <v>129</v>
+        <v>125</v>
       </c>
       <c r="B131" t="s">
-        <v>173</v>
+        <v>169</v>
       </c>
       <c r="C131" t="s">
-        <v>178</v>
+        <v>174</v>
       </c>
       <c r="D131" t="str">
         <f t="shared" ref="D131:D194" si="2">ROW(A130)&amp;".png"</f>
@@ -3090,13 +3102,13 @@
     </row>
     <row r="132" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A132" t="s">
-        <v>130</v>
+        <v>126</v>
       </c>
       <c r="B132" t="s">
-        <v>173</v>
+        <v>169</v>
       </c>
       <c r="C132" t="s">
-        <v>177</v>
+        <v>173</v>
       </c>
       <c r="D132" t="str">
         <f t="shared" si="2"/>
@@ -3105,13 +3117,13 @@
     </row>
     <row r="133" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A133" t="s">
-        <v>131</v>
+        <v>127</v>
       </c>
       <c r="B133" t="s">
-        <v>173</v>
+        <v>169</v>
       </c>
       <c r="C133" t="s">
-        <v>177</v>
+        <v>173</v>
       </c>
       <c r="D133" t="str">
         <f t="shared" si="2"/>
@@ -3120,13 +3132,13 @@
     </row>
     <row r="134" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A134" t="s">
-        <v>132</v>
+        <v>128</v>
       </c>
       <c r="B134" t="s">
-        <v>173</v>
+        <v>169</v>
       </c>
       <c r="C134" t="s">
-        <v>177</v>
+        <v>173</v>
       </c>
       <c r="D134" t="str">
         <f t="shared" si="2"/>
@@ -3135,13 +3147,13 @@
     </row>
     <row r="135" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A135" t="s">
-        <v>133</v>
+        <v>129</v>
       </c>
       <c r="B135" t="s">
-        <v>173</v>
+        <v>169</v>
       </c>
       <c r="C135" t="s">
-        <v>177</v>
+        <v>173</v>
       </c>
       <c r="D135" t="str">
         <f t="shared" si="2"/>
@@ -3150,13 +3162,13 @@
     </row>
     <row r="136" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A136" t="s">
-        <v>134</v>
+        <v>130</v>
       </c>
       <c r="B136" t="s">
-        <v>173</v>
+        <v>169</v>
       </c>
       <c r="C136" t="s">
-        <v>177</v>
+        <v>173</v>
       </c>
       <c r="D136" t="str">
         <f t="shared" si="2"/>
@@ -3165,13 +3177,13 @@
     </row>
     <row r="137" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A137" t="s">
-        <v>135</v>
+        <v>131</v>
       </c>
       <c r="B137" t="s">
-        <v>173</v>
+        <v>169</v>
       </c>
       <c r="C137" t="s">
-        <v>178</v>
+        <v>174</v>
       </c>
       <c r="D137" t="str">
         <f t="shared" si="2"/>
@@ -3180,13 +3192,13 @@
     </row>
     <row r="138" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A138" t="s">
-        <v>136</v>
+        <v>132</v>
       </c>
       <c r="B138" t="s">
-        <v>173</v>
+        <v>169</v>
       </c>
       <c r="C138" t="s">
-        <v>177</v>
+        <v>173</v>
       </c>
       <c r="D138" t="str">
         <f t="shared" si="2"/>
@@ -3195,13 +3207,13 @@
     </row>
     <row r="139" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A139" t="s">
-        <v>137</v>
+        <v>133</v>
       </c>
       <c r="B139" t="s">
-        <v>173</v>
+        <v>169</v>
       </c>
       <c r="C139" t="s">
-        <v>177</v>
+        <v>173</v>
       </c>
       <c r="D139" t="str">
         <f t="shared" si="2"/>
@@ -3210,13 +3222,13 @@
     </row>
     <row r="140" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A140" t="s">
-        <v>138</v>
+        <v>134</v>
       </c>
       <c r="B140" t="s">
-        <v>173</v>
+        <v>169</v>
       </c>
       <c r="C140" t="s">
-        <v>178</v>
+        <v>174</v>
       </c>
       <c r="D140" t="str">
         <f t="shared" si="2"/>
@@ -3225,13 +3237,13 @@
     </row>
     <row r="141" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A141" t="s">
-        <v>139</v>
+        <v>135</v>
       </c>
       <c r="B141" t="s">
-        <v>173</v>
+        <v>169</v>
       </c>
       <c r="C141" t="s">
-        <v>177</v>
+        <v>173</v>
       </c>
       <c r="D141" t="str">
         <f t="shared" si="2"/>
@@ -3240,13 +3252,13 @@
     </row>
     <row r="142" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A142" t="s">
-        <v>140</v>
+        <v>136</v>
       </c>
       <c r="B142" t="s">
-        <v>173</v>
+        <v>169</v>
       </c>
       <c r="C142" t="s">
-        <v>177</v>
+        <v>173</v>
       </c>
       <c r="D142" t="str">
         <f t="shared" si="2"/>
@@ -3255,13 +3267,13 @@
     </row>
     <row r="143" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A143" t="s">
-        <v>141</v>
+        <v>137</v>
       </c>
       <c r="B143" t="s">
-        <v>173</v>
+        <v>169</v>
       </c>
       <c r="C143" t="s">
-        <v>177</v>
+        <v>173</v>
       </c>
       <c r="D143" t="str">
         <f t="shared" si="2"/>
@@ -3270,13 +3282,13 @@
     </row>
     <row r="144" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A144" t="s">
-        <v>142</v>
+        <v>138</v>
       </c>
       <c r="B144" t="s">
-        <v>173</v>
+        <v>169</v>
       </c>
       <c r="C144" t="s">
-        <v>178</v>
+        <v>174</v>
       </c>
       <c r="D144" t="str">
         <f t="shared" si="2"/>
@@ -3285,13 +3297,13 @@
     </row>
     <row r="145" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A145" t="s">
-        <v>143</v>
+        <v>139</v>
       </c>
       <c r="B145" t="s">
-        <v>173</v>
+        <v>169</v>
       </c>
       <c r="C145" t="s">
-        <v>178</v>
+        <v>174</v>
       </c>
       <c r="D145" t="str">
         <f t="shared" si="2"/>
@@ -3300,13 +3312,13 @@
     </row>
     <row r="146" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A146" t="s">
-        <v>144</v>
+        <v>140</v>
       </c>
       <c r="B146" t="s">
-        <v>173</v>
+        <v>169</v>
       </c>
       <c r="C146" t="s">
-        <v>177</v>
+        <v>173</v>
       </c>
       <c r="D146" t="str">
         <f t="shared" si="2"/>
@@ -3315,13 +3327,13 @@
     </row>
     <row r="147" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A147" t="s">
-        <v>145</v>
+        <v>141</v>
       </c>
       <c r="B147" t="s">
-        <v>173</v>
+        <v>169</v>
       </c>
       <c r="C147" t="s">
-        <v>178</v>
+        <v>174</v>
       </c>
       <c r="D147" t="str">
         <f t="shared" si="2"/>
@@ -3330,13 +3342,13 @@
     </row>
     <row r="148" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A148" t="s">
-        <v>146</v>
+        <v>142</v>
       </c>
       <c r="B148" t="s">
-        <v>173</v>
+        <v>169</v>
       </c>
       <c r="C148" t="s">
-        <v>177</v>
+        <v>173</v>
       </c>
       <c r="D148" t="str">
         <f t="shared" si="2"/>
@@ -3345,13 +3357,13 @@
     </row>
     <row r="149" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A149" t="s">
-        <v>147</v>
+        <v>143</v>
       </c>
       <c r="B149" t="s">
-        <v>173</v>
+        <v>169</v>
       </c>
       <c r="C149" t="s">
-        <v>177</v>
+        <v>173</v>
       </c>
       <c r="D149" t="str">
         <f t="shared" si="2"/>
@@ -3360,13 +3372,13 @@
     </row>
     <row r="150" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A150" t="s">
-        <v>148</v>
+        <v>144</v>
       </c>
       <c r="B150" t="s">
-        <v>173</v>
+        <v>169</v>
       </c>
       <c r="C150" t="s">
-        <v>177</v>
+        <v>173</v>
       </c>
       <c r="D150" t="str">
         <f t="shared" si="2"/>
@@ -3375,13 +3387,13 @@
     </row>
     <row r="151" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A151" t="s">
-        <v>149</v>
+        <v>145</v>
       </c>
       <c r="B151" t="s">
-        <v>173</v>
+        <v>169</v>
       </c>
       <c r="C151" t="s">
-        <v>178</v>
+        <v>174</v>
       </c>
       <c r="D151" t="str">
         <f t="shared" si="2"/>
@@ -3390,13 +3402,13 @@
     </row>
     <row r="152" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A152" t="s">
-        <v>150</v>
+        <v>146</v>
       </c>
       <c r="B152" t="s">
-        <v>173</v>
+        <v>169</v>
       </c>
       <c r="C152" t="s">
-        <v>178</v>
+        <v>174</v>
       </c>
       <c r="D152" t="str">
         <f t="shared" si="2"/>
@@ -3405,13 +3417,13 @@
     </row>
     <row r="153" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A153" t="s">
-        <v>151</v>
+        <v>147</v>
       </c>
       <c r="B153" t="s">
-        <v>173</v>
+        <v>169</v>
       </c>
       <c r="C153" t="s">
-        <v>178</v>
+        <v>174</v>
       </c>
       <c r="D153" t="str">
         <f t="shared" si="2"/>
@@ -3420,13 +3432,13 @@
     </row>
     <row r="154" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A154" t="s">
-        <v>152</v>
+        <v>148</v>
       </c>
       <c r="B154" t="s">
-        <v>173</v>
+        <v>169</v>
       </c>
       <c r="C154" t="s">
-        <v>178</v>
+        <v>174</v>
       </c>
       <c r="D154" t="str">
         <f t="shared" si="2"/>
@@ -3435,13 +3447,13 @@
     </row>
     <row r="155" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A155" t="s">
-        <v>153</v>
+        <v>149</v>
       </c>
       <c r="B155" t="s">
-        <v>173</v>
+        <v>169</v>
       </c>
       <c r="C155" t="s">
-        <v>178</v>
+        <v>174</v>
       </c>
       <c r="D155" t="str">
         <f t="shared" si="2"/>
@@ -3450,13 +3462,13 @@
     </row>
     <row r="156" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A156" t="s">
-        <v>154</v>
+        <v>150</v>
       </c>
       <c r="B156" t="s">
-        <v>173</v>
+        <v>169</v>
       </c>
       <c r="C156" t="s">
-        <v>177</v>
+        <v>173</v>
       </c>
       <c r="D156" t="str">
         <f t="shared" si="2"/>
@@ -3465,13 +3477,13 @@
     </row>
     <row r="157" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A157" t="s">
-        <v>155</v>
+        <v>151</v>
       </c>
       <c r="B157" t="s">
-        <v>173</v>
+        <v>169</v>
       </c>
       <c r="C157" t="s">
-        <v>178</v>
+        <v>174</v>
       </c>
       <c r="D157" t="str">
         <f t="shared" si="2"/>
@@ -3480,13 +3492,13 @@
     </row>
     <row r="158" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A158" t="s">
-        <v>156</v>
+        <v>152</v>
       </c>
       <c r="B158" t="s">
-        <v>173</v>
+        <v>169</v>
       </c>
       <c r="C158" t="s">
-        <v>178</v>
+        <v>174</v>
       </c>
       <c r="D158" t="str">
         <f t="shared" si="2"/>
@@ -3495,13 +3507,13 @@
     </row>
     <row r="159" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A159" t="s">
-        <v>157</v>
+        <v>153</v>
       </c>
       <c r="B159" t="s">
-        <v>173</v>
+        <v>169</v>
       </c>
       <c r="C159" t="s">
-        <v>178</v>
+        <v>174</v>
       </c>
       <c r="D159" t="str">
         <f t="shared" si="2"/>
@@ -3510,13 +3522,13 @@
     </row>
     <row r="160" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A160" t="s">
-        <v>158</v>
+        <v>154</v>
       </c>
       <c r="B160" t="s">
-        <v>173</v>
+        <v>169</v>
       </c>
       <c r="C160" t="s">
-        <v>177</v>
+        <v>173</v>
       </c>
       <c r="D160" t="str">
         <f t="shared" si="2"/>
@@ -3525,13 +3537,13 @@
     </row>
     <row r="161" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A161" t="s">
-        <v>159</v>
+        <v>155</v>
       </c>
       <c r="B161" t="s">
-        <v>173</v>
+        <v>169</v>
       </c>
       <c r="C161" t="s">
-        <v>177</v>
+        <v>173</v>
       </c>
       <c r="D161" t="str">
         <f t="shared" si="2"/>
@@ -3540,13 +3552,13 @@
     </row>
     <row r="162" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A162" t="s">
-        <v>160</v>
+        <v>156</v>
       </c>
       <c r="B162" t="s">
-        <v>173</v>
+        <v>169</v>
       </c>
       <c r="C162" t="s">
-        <v>177</v>
+        <v>173</v>
       </c>
       <c r="D162" t="str">
         <f t="shared" si="2"/>
@@ -3555,13 +3567,13 @@
     </row>
     <row r="163" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A163" t="s">
-        <v>161</v>
+        <v>157</v>
       </c>
       <c r="B163" t="s">
-        <v>173</v>
+        <v>169</v>
       </c>
       <c r="C163" t="s">
-        <v>178</v>
+        <v>174</v>
       </c>
       <c r="D163" t="str">
         <f t="shared" si="2"/>
@@ -3570,13 +3582,13 @@
     </row>
     <row r="164" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A164" t="s">
-        <v>162</v>
+        <v>158</v>
       </c>
       <c r="B164" t="s">
-        <v>173</v>
+        <v>169</v>
       </c>
       <c r="C164" t="s">
-        <v>177</v>
+        <v>173</v>
       </c>
       <c r="D164" t="str">
         <f t="shared" si="2"/>
@@ -3585,13 +3597,13 @@
     </row>
     <row r="165" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A165" t="s">
-        <v>163</v>
+        <v>159</v>
       </c>
       <c r="B165" t="s">
-        <v>173</v>
+        <v>169</v>
       </c>
       <c r="C165" t="s">
-        <v>177</v>
+        <v>173</v>
       </c>
       <c r="D165" t="str">
         <f t="shared" si="2"/>
@@ -3600,13 +3612,13 @@
     </row>
     <row r="166" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A166" t="s">
-        <v>164</v>
+        <v>160</v>
       </c>
       <c r="B166" t="s">
-        <v>173</v>
+        <v>169</v>
       </c>
       <c r="C166" t="s">
-        <v>178</v>
+        <v>174</v>
       </c>
       <c r="D166" t="str">
         <f t="shared" si="2"/>
@@ -3615,13 +3627,13 @@
     </row>
     <row r="167" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A167" t="s">
-        <v>165</v>
+        <v>161</v>
       </c>
       <c r="B167" t="s">
-        <v>173</v>
+        <v>169</v>
       </c>
       <c r="C167" t="s">
-        <v>178</v>
+        <v>174</v>
       </c>
       <c r="D167" t="str">
         <f t="shared" si="2"/>
@@ -3630,13 +3642,13 @@
     </row>
     <row r="168" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A168" t="s">
-        <v>166</v>
+        <v>162</v>
       </c>
       <c r="B168" t="s">
-        <v>173</v>
+        <v>169</v>
       </c>
       <c r="C168" t="s">
-        <v>178</v>
+        <v>174</v>
       </c>
       <c r="D168" t="str">
         <f t="shared" si="2"/>
@@ -3645,13 +3657,13 @@
     </row>
     <row r="169" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A169" t="s">
-        <v>167</v>
+        <v>163</v>
       </c>
       <c r="B169" t="s">
-        <v>173</v>
+        <v>169</v>
       </c>
       <c r="C169" t="s">
-        <v>178</v>
+        <v>174</v>
       </c>
       <c r="D169" t="str">
         <f t="shared" si="2"/>
@@ -3660,13 +3672,13 @@
     </row>
     <row r="170" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A170" t="s">
-        <v>168</v>
+        <v>164</v>
       </c>
       <c r="B170" t="s">
-        <v>173</v>
+        <v>169</v>
       </c>
       <c r="C170" t="s">
-        <v>178</v>
+        <v>174</v>
       </c>
       <c r="D170" t="str">
         <f t="shared" si="2"/>
@@ -3675,13 +3687,13 @@
     </row>
     <row r="171" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A171" t="s">
-        <v>169</v>
+        <v>165</v>
       </c>
       <c r="B171" t="s">
-        <v>173</v>
+        <v>169</v>
       </c>
       <c r="C171" t="s">
-        <v>178</v>
+        <v>174</v>
       </c>
       <c r="D171" t="str">
         <f t="shared" si="2"/>
@@ -3690,13 +3702,13 @@
     </row>
     <row r="172" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A172" t="s">
-        <v>170</v>
+        <v>166</v>
       </c>
       <c r="B172" t="s">
-        <v>173</v>
+        <v>169</v>
       </c>
       <c r="C172" t="s">
-        <v>178</v>
+        <v>173</v>
       </c>
       <c r="D172" t="str">
         <f t="shared" si="2"/>
@@ -3705,13 +3717,13 @@
     </row>
     <row r="173" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A173" t="s">
-        <v>171</v>
+        <v>167</v>
       </c>
       <c r="B173" t="s">
-        <v>173</v>
+        <v>169</v>
       </c>
       <c r="C173" t="s">
-        <v>177</v>
+        <v>173</v>
       </c>
       <c r="D173" t="str">
         <f t="shared" si="2"/>
@@ -3720,13 +3732,13 @@
     </row>
     <row r="174" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A174" t="s">
-        <v>172</v>
+        <v>168</v>
       </c>
       <c r="B174" t="s">
-        <v>173</v>
+        <v>169</v>
       </c>
       <c r="C174" t="s">
-        <v>177</v>
+        <v>173</v>
       </c>
       <c r="D174" t="str">
         <f t="shared" si="2"/>
@@ -3735,13 +3747,13 @@
     </row>
     <row r="175" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A175" t="s">
-        <v>180</v>
+        <v>176</v>
       </c>
       <c r="B175" s="2" t="s">
-        <v>229</v>
+        <v>225</v>
       </c>
       <c r="C175" t="s">
-        <v>177</v>
+        <v>173</v>
       </c>
       <c r="D175" t="str">
         <f t="shared" si="2"/>
@@ -3750,13 +3762,13 @@
     </row>
     <row r="176" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A176" t="s">
-        <v>181</v>
+        <v>177</v>
       </c>
       <c r="B176" s="2" t="s">
-        <v>229</v>
+        <v>225</v>
       </c>
       <c r="C176" t="s">
-        <v>177</v>
+        <v>173</v>
       </c>
       <c r="D176" t="str">
         <f t="shared" si="2"/>
@@ -3765,13 +3777,13 @@
     </row>
     <row r="177" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A177" t="s">
-        <v>182</v>
+        <v>178</v>
       </c>
       <c r="B177" s="2" t="s">
-        <v>229</v>
+        <v>225</v>
       </c>
       <c r="C177" t="s">
-        <v>177</v>
+        <v>173</v>
       </c>
       <c r="D177" t="str">
         <f t="shared" si="2"/>
@@ -3780,13 +3792,13 @@
     </row>
     <row r="178" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A178" t="s">
-        <v>183</v>
+        <v>179</v>
       </c>
       <c r="B178" s="2" t="s">
-        <v>229</v>
+        <v>225</v>
       </c>
       <c r="C178" t="s">
-        <v>177</v>
+        <v>173</v>
       </c>
       <c r="D178" t="str">
         <f t="shared" si="2"/>
@@ -3795,13 +3807,13 @@
     </row>
     <row r="179" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A179" t="s">
-        <v>184</v>
+        <v>180</v>
       </c>
       <c r="B179" s="2" t="s">
-        <v>229</v>
+        <v>225</v>
       </c>
       <c r="C179" t="s">
-        <v>177</v>
+        <v>173</v>
       </c>
       <c r="D179" t="str">
         <f t="shared" si="2"/>
@@ -3810,13 +3822,13 @@
     </row>
     <row r="180" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A180" t="s">
-        <v>185</v>
+        <v>181</v>
       </c>
       <c r="B180" s="2" t="s">
-        <v>229</v>
+        <v>225</v>
       </c>
       <c r="C180" t="s">
-        <v>177</v>
+        <v>173</v>
       </c>
       <c r="D180" t="str">
         <f t="shared" si="2"/>
@@ -3825,13 +3837,13 @@
     </row>
     <row r="181" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A181" t="s">
-        <v>186</v>
+        <v>182</v>
       </c>
       <c r="B181" s="2" t="s">
-        <v>229</v>
+        <v>225</v>
       </c>
       <c r="C181" t="s">
-        <v>177</v>
+        <v>173</v>
       </c>
       <c r="D181" t="str">
         <f t="shared" si="2"/>
@@ -3840,13 +3852,13 @@
     </row>
     <row r="182" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A182" t="s">
-        <v>187</v>
+        <v>183</v>
       </c>
       <c r="B182" s="2" t="s">
-        <v>229</v>
+        <v>225</v>
       </c>
       <c r="C182" t="s">
-        <v>177</v>
+        <v>173</v>
       </c>
       <c r="D182" t="str">
         <f t="shared" si="2"/>
@@ -3855,13 +3867,13 @@
     </row>
     <row r="183" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A183" t="s">
-        <v>188</v>
+        <v>184</v>
       </c>
       <c r="B183" s="2" t="s">
-        <v>229</v>
+        <v>225</v>
       </c>
       <c r="C183" t="s">
-        <v>177</v>
+        <v>173</v>
       </c>
       <c r="D183" t="str">
         <f t="shared" si="2"/>
@@ -3870,13 +3882,13 @@
     </row>
     <row r="184" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A184" t="s">
-        <v>189</v>
+        <v>185</v>
       </c>
       <c r="B184" s="2" t="s">
-        <v>229</v>
+        <v>225</v>
       </c>
       <c r="C184" t="s">
-        <v>177</v>
+        <v>173</v>
       </c>
       <c r="D184" t="str">
         <f t="shared" si="2"/>
@@ -3885,13 +3897,13 @@
     </row>
     <row r="185" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A185" t="s">
-        <v>190</v>
+        <v>186</v>
       </c>
       <c r="B185" s="2" t="s">
-        <v>229</v>
+        <v>225</v>
       </c>
       <c r="C185" t="s">
-        <v>177</v>
+        <v>173</v>
       </c>
       <c r="D185" t="str">
         <f t="shared" si="2"/>
@@ -3900,13 +3912,13 @@
     </row>
     <row r="186" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A186" t="s">
-        <v>191</v>
+        <v>187</v>
       </c>
       <c r="B186" s="2" t="s">
-        <v>229</v>
+        <v>225</v>
       </c>
       <c r="C186" t="s">
-        <v>177</v>
+        <v>173</v>
       </c>
       <c r="D186" t="str">
         <f t="shared" si="2"/>
@@ -3915,13 +3927,13 @@
     </row>
     <row r="187" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A187" t="s">
-        <v>192</v>
+        <v>188</v>
       </c>
       <c r="B187" s="2" t="s">
-        <v>229</v>
+        <v>225</v>
       </c>
       <c r="C187" t="s">
-        <v>177</v>
+        <v>173</v>
       </c>
       <c r="D187" t="str">
         <f t="shared" si="2"/>
@@ -3930,13 +3942,13 @@
     </row>
     <row r="188" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A188" t="s">
-        <v>193</v>
+        <v>189</v>
       </c>
       <c r="B188" s="2" t="s">
-        <v>229</v>
+        <v>225</v>
       </c>
       <c r="C188" t="s">
-        <v>177</v>
+        <v>173</v>
       </c>
       <c r="D188" t="str">
         <f t="shared" si="2"/>
@@ -3945,13 +3957,13 @@
     </row>
     <row r="189" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A189" t="s">
-        <v>194</v>
+        <v>190</v>
       </c>
       <c r="B189" s="2" t="s">
-        <v>229</v>
+        <v>225</v>
       </c>
       <c r="C189" t="s">
-        <v>177</v>
+        <v>173</v>
       </c>
       <c r="D189" t="str">
         <f t="shared" si="2"/>
@@ -3960,13 +3972,13 @@
     </row>
     <row r="190" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A190" t="s">
-        <v>195</v>
+        <v>191</v>
       </c>
       <c r="B190" s="2" t="s">
-        <v>229</v>
+        <v>225</v>
       </c>
       <c r="C190" t="s">
-        <v>177</v>
+        <v>173</v>
       </c>
       <c r="D190" t="str">
         <f t="shared" si="2"/>
@@ -3975,13 +3987,13 @@
     </row>
     <row r="191" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A191" t="s">
-        <v>196</v>
+        <v>192</v>
       </c>
       <c r="B191" s="2" t="s">
-        <v>229</v>
+        <v>225</v>
       </c>
       <c r="C191" t="s">
-        <v>177</v>
+        <v>173</v>
       </c>
       <c r="D191" t="str">
         <f t="shared" si="2"/>
@@ -3990,13 +4002,13 @@
     </row>
     <row r="192" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A192" t="s">
-        <v>197</v>
+        <v>193</v>
       </c>
       <c r="B192" s="2" t="s">
-        <v>229</v>
+        <v>225</v>
       </c>
       <c r="C192" t="s">
-        <v>177</v>
+        <v>173</v>
       </c>
       <c r="D192" t="str">
         <f t="shared" si="2"/>
@@ -4005,13 +4017,13 @@
     </row>
     <row r="193" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A193" t="s">
-        <v>198</v>
+        <v>194</v>
       </c>
       <c r="B193" s="2" t="s">
-        <v>229</v>
+        <v>225</v>
       </c>
       <c r="C193" t="s">
-        <v>177</v>
+        <v>173</v>
       </c>
       <c r="D193" t="str">
         <f t="shared" si="2"/>
@@ -4020,13 +4032,13 @@
     </row>
     <row r="194" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A194" t="s">
-        <v>199</v>
+        <v>195</v>
       </c>
       <c r="B194" s="2" t="s">
-        <v>229</v>
+        <v>225</v>
       </c>
       <c r="C194" t="s">
-        <v>177</v>
+        <v>173</v>
       </c>
       <c r="D194" t="str">
         <f t="shared" si="2"/>
@@ -4035,13 +4047,13 @@
     </row>
     <row r="195" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A195" t="s">
-        <v>200</v>
+        <v>196</v>
       </c>
       <c r="B195" s="2" t="s">
-        <v>229</v>
+        <v>225</v>
       </c>
       <c r="C195" t="s">
-        <v>177</v>
+        <v>173</v>
       </c>
       <c r="D195" t="str">
         <f t="shared" ref="D195:D223" si="3">ROW(A194)&amp;".png"</f>
@@ -4050,13 +4062,13 @@
     </row>
     <row r="196" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A196" t="s">
-        <v>201</v>
+        <v>197</v>
       </c>
       <c r="B196" s="2" t="s">
-        <v>229</v>
+        <v>225</v>
       </c>
       <c r="C196" t="s">
-        <v>177</v>
+        <v>173</v>
       </c>
       <c r="D196" t="str">
         <f t="shared" si="3"/>
@@ -4065,13 +4077,13 @@
     </row>
     <row r="197" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A197" t="s">
-        <v>202</v>
+        <v>198</v>
       </c>
       <c r="B197" s="2" t="s">
-        <v>229</v>
+        <v>225</v>
       </c>
       <c r="C197" t="s">
-        <v>177</v>
+        <v>173</v>
       </c>
       <c r="D197" t="str">
         <f t="shared" si="3"/>
@@ -4080,13 +4092,13 @@
     </row>
     <row r="198" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A198" t="s">
-        <v>203</v>
+        <v>199</v>
       </c>
       <c r="B198" s="2" t="s">
-        <v>229</v>
+        <v>225</v>
       </c>
       <c r="C198" t="s">
-        <v>177</v>
+        <v>173</v>
       </c>
       <c r="D198" t="str">
         <f t="shared" si="3"/>
@@ -4095,13 +4107,13 @@
     </row>
     <row r="199" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A199" t="s">
-        <v>204</v>
+        <v>200</v>
       </c>
       <c r="B199" s="2" t="s">
-        <v>229</v>
+        <v>225</v>
       </c>
       <c r="C199" t="s">
-        <v>177</v>
+        <v>173</v>
       </c>
       <c r="D199" t="str">
         <f t="shared" si="3"/>
@@ -4110,13 +4122,13 @@
     </row>
     <row r="200" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A200" t="s">
-        <v>205</v>
+        <v>201</v>
       </c>
       <c r="B200" s="2" t="s">
-        <v>229</v>
+        <v>225</v>
       </c>
       <c r="C200" t="s">
-        <v>177</v>
+        <v>173</v>
       </c>
       <c r="D200" t="str">
         <f t="shared" si="3"/>
@@ -4125,13 +4137,13 @@
     </row>
     <row r="201" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A201" t="s">
-        <v>206</v>
+        <v>202</v>
       </c>
       <c r="B201" s="2" t="s">
-        <v>229</v>
+        <v>225</v>
       </c>
       <c r="C201" t="s">
-        <v>177</v>
+        <v>173</v>
       </c>
       <c r="D201" t="str">
         <f t="shared" si="3"/>
@@ -4140,13 +4152,13 @@
     </row>
     <row r="202" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A202" t="s">
-        <v>207</v>
+        <v>203</v>
       </c>
       <c r="B202" s="2" t="s">
-        <v>229</v>
+        <v>225</v>
       </c>
       <c r="C202" t="s">
-        <v>177</v>
+        <v>173</v>
       </c>
       <c r="D202" t="str">
         <f t="shared" si="3"/>
@@ -4155,13 +4167,13 @@
     </row>
     <row r="203" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A203" t="s">
-        <v>208</v>
+        <v>204</v>
       </c>
       <c r="B203" s="2" t="s">
-        <v>229</v>
+        <v>225</v>
       </c>
       <c r="C203" t="s">
-        <v>177</v>
+        <v>173</v>
       </c>
       <c r="D203" t="str">
         <f t="shared" si="3"/>
@@ -4170,13 +4182,13 @@
     </row>
     <row r="204" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A204" t="s">
-        <v>209</v>
+        <v>205</v>
       </c>
       <c r="B204" s="2" t="s">
-        <v>229</v>
+        <v>225</v>
       </c>
       <c r="C204" t="s">
-        <v>177</v>
+        <v>173</v>
       </c>
       <c r="D204" t="str">
         <f t="shared" si="3"/>
@@ -4185,13 +4197,13 @@
     </row>
     <row r="205" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A205" t="s">
-        <v>210</v>
+        <v>206</v>
       </c>
       <c r="B205" s="2" t="s">
-        <v>229</v>
+        <v>225</v>
       </c>
       <c r="C205" t="s">
-        <v>177</v>
+        <v>173</v>
       </c>
       <c r="D205" t="str">
         <f t="shared" si="3"/>
@@ -4200,13 +4212,13 @@
     </row>
     <row r="206" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A206" t="s">
-        <v>211</v>
+        <v>207</v>
       </c>
       <c r="B206" s="2" t="s">
-        <v>229</v>
+        <v>225</v>
       </c>
       <c r="C206" t="s">
-        <v>177</v>
+        <v>173</v>
       </c>
       <c r="D206" t="str">
         <f t="shared" si="3"/>
@@ -4215,13 +4227,13 @@
     </row>
     <row r="207" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A207" t="s">
-        <v>212</v>
+        <v>208</v>
       </c>
       <c r="B207" s="2" t="s">
-        <v>229</v>
+        <v>225</v>
       </c>
       <c r="C207" t="s">
-        <v>177</v>
+        <v>173</v>
       </c>
       <c r="D207" t="str">
         <f t="shared" si="3"/>
@@ -4230,13 +4242,13 @@
     </row>
     <row r="208" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A208" t="s">
-        <v>213</v>
+        <v>209</v>
       </c>
       <c r="B208" s="2" t="s">
-        <v>229</v>
+        <v>225</v>
       </c>
       <c r="C208" t="s">
-        <v>177</v>
+        <v>173</v>
       </c>
       <c r="D208" t="str">
         <f t="shared" si="3"/>
@@ -4245,13 +4257,13 @@
     </row>
     <row r="209" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A209" t="s">
-        <v>214</v>
+        <v>210</v>
       </c>
       <c r="B209" s="2" t="s">
-        <v>229</v>
+        <v>225</v>
       </c>
       <c r="C209" t="s">
-        <v>177</v>
+        <v>173</v>
       </c>
       <c r="D209" t="str">
         <f t="shared" si="3"/>
@@ -4260,13 +4272,13 @@
     </row>
     <row r="210" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A210" t="s">
-        <v>215</v>
+        <v>211</v>
       </c>
       <c r="B210" s="2" t="s">
-        <v>229</v>
+        <v>225</v>
       </c>
       <c r="C210" t="s">
-        <v>177</v>
+        <v>173</v>
       </c>
       <c r="D210" t="str">
         <f t="shared" si="3"/>
@@ -4275,13 +4287,13 @@
     </row>
     <row r="211" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A211" t="s">
-        <v>216</v>
+        <v>212</v>
       </c>
       <c r="B211" s="2" t="s">
-        <v>229</v>
+        <v>225</v>
       </c>
       <c r="C211" t="s">
-        <v>177</v>
+        <v>173</v>
       </c>
       <c r="D211" t="str">
         <f t="shared" si="3"/>
@@ -4290,13 +4302,13 @@
     </row>
     <row r="212" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A212" t="s">
-        <v>217</v>
+        <v>213</v>
       </c>
       <c r="B212" s="2" t="s">
-        <v>229</v>
+        <v>225</v>
       </c>
       <c r="C212" t="s">
-        <v>177</v>
+        <v>173</v>
       </c>
       <c r="D212" t="str">
         <f t="shared" si="3"/>
@@ -4305,13 +4317,13 @@
     </row>
     <row r="213" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A213" t="s">
-        <v>218</v>
+        <v>214</v>
       </c>
       <c r="B213" s="2" t="s">
-        <v>229</v>
+        <v>225</v>
       </c>
       <c r="C213" t="s">
-        <v>177</v>
+        <v>173</v>
       </c>
       <c r="D213" t="str">
         <f t="shared" si="3"/>
@@ -4320,13 +4332,13 @@
     </row>
     <row r="214" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A214" t="s">
-        <v>219</v>
+        <v>215</v>
       </c>
       <c r="B214" s="2" t="s">
-        <v>229</v>
+        <v>225</v>
       </c>
       <c r="C214" t="s">
-        <v>177</v>
+        <v>173</v>
       </c>
       <c r="D214" t="str">
         <f t="shared" si="3"/>
@@ -4335,13 +4347,13 @@
     </row>
     <row r="215" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A215" t="s">
-        <v>220</v>
+        <v>216</v>
       </c>
       <c r="B215" s="2" t="s">
-        <v>229</v>
+        <v>225</v>
       </c>
       <c r="C215" t="s">
-        <v>177</v>
+        <v>173</v>
       </c>
       <c r="D215" t="str">
         <f t="shared" si="3"/>
@@ -4350,13 +4362,13 @@
     </row>
     <row r="216" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A216" t="s">
-        <v>221</v>
+        <v>217</v>
       </c>
       <c r="B216" s="2" t="s">
-        <v>229</v>
+        <v>225</v>
       </c>
       <c r="C216" t="s">
-        <v>177</v>
+        <v>173</v>
       </c>
       <c r="D216" t="str">
         <f t="shared" si="3"/>
@@ -4365,13 +4377,13 @@
     </row>
     <row r="217" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A217" t="s">
-        <v>222</v>
+        <v>218</v>
       </c>
       <c r="B217" s="2" t="s">
-        <v>229</v>
+        <v>225</v>
       </c>
       <c r="C217" t="s">
-        <v>177</v>
+        <v>173</v>
       </c>
       <c r="D217" t="str">
         <f t="shared" si="3"/>
@@ -4380,13 +4392,13 @@
     </row>
     <row r="218" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A218" t="s">
-        <v>223</v>
+        <v>219</v>
       </c>
       <c r="B218" s="2" t="s">
-        <v>229</v>
+        <v>225</v>
       </c>
       <c r="C218" t="s">
-        <v>177</v>
+        <v>173</v>
       </c>
       <c r="D218" t="str">
         <f t="shared" si="3"/>
@@ -4395,13 +4407,13 @@
     </row>
     <row r="219" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A219" t="s">
-        <v>224</v>
+        <v>220</v>
       </c>
       <c r="B219" s="2" t="s">
-        <v>229</v>
+        <v>225</v>
       </c>
       <c r="C219" t="s">
-        <v>177</v>
+        <v>173</v>
       </c>
       <c r="D219" t="str">
         <f t="shared" si="3"/>
@@ -4410,13 +4422,13 @@
     </row>
     <row r="220" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A220" t="s">
-        <v>225</v>
+        <v>221</v>
       </c>
       <c r="B220" s="2" t="s">
-        <v>229</v>
+        <v>225</v>
       </c>
       <c r="C220" t="s">
-        <v>177</v>
+        <v>173</v>
       </c>
       <c r="D220" t="str">
         <f t="shared" si="3"/>
@@ -4425,13 +4437,13 @@
     </row>
     <row r="221" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A221" t="s">
-        <v>226</v>
+        <v>222</v>
       </c>
       <c r="B221" s="2" t="s">
-        <v>229</v>
+        <v>225</v>
       </c>
       <c r="C221" t="s">
-        <v>177</v>
+        <v>173</v>
       </c>
       <c r="D221" t="str">
         <f t="shared" si="3"/>
@@ -4440,13 +4452,13 @@
     </row>
     <row r="222" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A222" t="s">
-        <v>227</v>
+        <v>223</v>
       </c>
       <c r="B222" s="2" t="s">
-        <v>229</v>
+        <v>225</v>
       </c>
       <c r="C222" t="s">
-        <v>177</v>
+        <v>173</v>
       </c>
       <c r="D222" t="str">
         <f t="shared" si="3"/>
@@ -4455,17 +4467,45 @@
     </row>
     <row r="223" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A223" t="s">
-        <v>228</v>
+        <v>224</v>
       </c>
       <c r="B223" s="2" t="s">
-        <v>229</v>
+        <v>225</v>
       </c>
       <c r="C223" t="s">
-        <v>177</v>
+        <v>173</v>
       </c>
       <c r="D223" t="str">
         <f t="shared" si="3"/>
         <v>222.png</v>
+      </c>
+    </row>
+    <row r="224" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A224" t="s">
+        <v>229</v>
+      </c>
+      <c r="B224" s="2" t="s">
+        <v>225</v>
+      </c>
+      <c r="C224" t="s">
+        <v>173</v>
+      </c>
+      <c r="D224" t="s">
+        <v>230</v>
+      </c>
+    </row>
+    <row r="225" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A225" t="s">
+        <v>231</v>
+      </c>
+      <c r="B225" s="2" t="s">
+        <v>225</v>
+      </c>
+      <c r="C225" t="s">
+        <v>173</v>
+      </c>
+      <c r="D225" t="s">
+        <v>232</v>
       </c>
     </row>
   </sheetData>

</xml_diff>